<commit_message>
read data from excel
</commit_message>
<xml_diff>
--- a/data/testdata.xlsx
+++ b/data/testdata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Course\Playwright_typescript\PlaywrightJuly2026\TDDFramework\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Course\Playwright_typescript\PlaywrightJuly2026\PlaywrightCucumberFramework_July26\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79225FA-DF0D-4F72-939F-26880071A867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{994223B9-46F3-4C90-99B4-3C8F1888BE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>TestCase</t>
   </si>
@@ -36,34 +36,19 @@
     <t>password</t>
   </si>
   <si>
-    <t>TC01</t>
-  </si>
-  <si>
     <t>admin</t>
   </si>
   <si>
     <t>admin123</t>
   </si>
   <si>
-    <t>TC02</t>
-  </si>
-  <si>
-    <t>TC03</t>
-  </si>
-  <si>
-    <t>TC04</t>
-  </si>
-  <si>
-    <t>invaliduser</t>
-  </si>
-  <si>
-    <t>TC05</t>
-  </si>
-  <si>
-    <t>invalidpassword</t>
-  </si>
-  <si>
-    <t>TC06</t>
+    <t>TC01_valid_login</t>
+  </si>
+  <si>
+    <t>TC02_Invalid_login</t>
+  </si>
+  <si>
+    <t>admin123455</t>
   </si>
 </sst>
 </file>
@@ -122,11 +107,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -413,7 +395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.06640625" customWidth="1"/>
@@ -422,75 +404,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>